<commit_message>
Responsive design, profile redesign, UI fixes, attendance validation, button theming
- Full responsive CSS (mobile/tablet breakpoints)
- Profile hero card with gradient banner + career quote
- All buttons use company theme (fixed email domain detection)
- Attendance request: checkout date auto-syncs, validates late shifts
- Data Entry: removed employee project creation
- Time Sheet: summary stats card, status tags, GTL gap warning
- Dashboard: team-filtered attendance, removed check-in/out
- Leaves: merged apply into single page with leave type info
- My Attendance: summary stats, checkout request button
- Swagger: 124 endpoints documented with examples

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Sprint_Plan_Abdul_Mannan.xlsx
+++ b/docs/Sprint_Plan_Abdul_Mannan.xlsx
@@ -1,10 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="20417"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30CBA383-1DB1-4454-8ABA-521A0B0004A6}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Sprint Plan" state="visible" r:id="rId4"/>
+    <sheet name="Sprint Plan" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
@@ -46,9 +50,6 @@
     <t>Thu 03 Apr</t>
   </si>
   <si>
-    <t>Create Swagger, Org. charts, few minor tweaks</t>
-  </si>
-  <si>
     <t>Fri 04 Apr</t>
   </si>
   <si>
@@ -116,43 +117,51 @@
   </si>
   <si>
     <t>Full testing with real users — employee login, lead approval, admin management. Get sign-off for go-live</t>
+  </si>
+  <si>
+    <t>Create Swagger, Org. charts, few minor tweaks, add responsiveness</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="6" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <color rgb="FFFFFF"/>
       <sz val="11"/>
+      <color rgb="FF154360"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF333333"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <color rgb="154360"/>
       <sz val="11"/>
-    </font>
-    <font>
-      <color rgb="333333"/>
-      <sz val="11"/>
+      <color rgb="FF389E0D"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <color rgb="389E0D"/>
       <sz val="11"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="D48806"/>
-      <sz val="11"/>
+      <color rgb="FFD48806"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="7">
@@ -164,27 +173,27 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="154360"/>
+        <fgColor rgb="FF154360"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="F0F7FF"/>
+        <fgColor rgb="FFF0F7FF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="F6FFED"/>
+        <fgColor rgb="FFF6FFED"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF"/>
+        <fgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF7E6"/>
+        <fgColor rgb="FFFFF7E6"/>
       </patternFill>
     </fill>
   </fills>
@@ -201,7 +210,7 @@
       <right/>
       <top/>
       <bottom style="thin">
-        <color rgb="E0E0E0"/>
+        <color rgb="FFE0E0E0"/>
       </bottom>
       <diagonal/>
     </border>
@@ -570,19 +579,19 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
-    <tabColor rgb="154360"/>
+    <tabColor rgb="FF154360"/>
   </sheetPr>
   <dimension ref="A1:C16"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
     <col min="2" max="2" width="90" customWidth="1"/>
     <col min="3" max="3" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="24" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -593,7 +602,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" ht="32" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>3</v>
       </c>
@@ -604,7 +613,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" ht="32" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>6</v>
       </c>
@@ -615,7 +624,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" ht="32" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>8</v>
       </c>
@@ -626,140 +635,140 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" ht="32" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>10</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="6" ht="32" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="C6" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="C6" s="4" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="7" ht="32" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="5" t="s">
+      <c r="B7" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="C7" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C7" s="4" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="8" ht="32" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
+      <c r="B8" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B8" s="3" t="s">
-        <v>17</v>
-      </c>
       <c r="C8" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="5" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="9" ht="32" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="5" t="s">
+      <c r="B9" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="C9" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="C9" s="7" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="10" ht="32" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
+      <c r="B10" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="C10" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="C10" s="7" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="11" ht="32" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" s="5" t="s">
+      <c r="B11" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="C11" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C11" s="7" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="12" ht="32" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
+      <c r="B12" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="C12" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="C12" s="7" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="13" ht="32" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="5" t="s">
+      <c r="B13" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="B13" s="6" t="s">
+      <c r="C13" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="C13" s="7" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="14" ht="32" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" s="2" t="s">
+      <c r="B14" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="C14" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="C14" s="7" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="15" ht="32" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" s="5" t="s">
+      <c r="B15" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="B15" s="6" t="s">
+      <c r="C15" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C15" s="7" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="16" ht="32" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" s="2" t="s">
+      <c r="B16" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="B16" s="3" t="s">
-        <v>34</v>
-      </c>
       <c r="C16" s="7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>